<commit_message>
📊 Horarios actualizados Línea 141 - 1901
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-24.xlsx
+++ b/data/horarios-141-2026-03-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:46:40</t>
+          <t>Última actualización: 02:48:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -473,12 +473,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>01:46:40</t>
+          <t>02:48:19</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:01</t>
+          <t>03:02</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>75</v>
+        <v>14</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,23 +498,48 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>01:46:40</t>
+          <t>02:48:19</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:02</t>
+          <t>03:48</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>02:48:19</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>04:02</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>74</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -544,7 +569,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:46:40</t>
+          <t>Última actualización: 02:48:19</t>
         </is>
       </c>
     </row>
@@ -579,7 +604,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:46:40</t>
+          <t>Última actualización: 02:48:19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1902
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-24.xlsx
+++ b/data/horarios-141-2026-03-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:48:19</t>
+          <t>Última actualización: 03:45:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:48:19</t>
+          <t>03:45:20</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:02</t>
+          <t>03:48</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>02:48:19</t>
+          <t>03:45:20</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>04:02</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>60</v>
+        <v>17</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,12 +523,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>02:48:19</t>
+          <t>03:45:20</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04:02</t>
+          <t>04:48</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -537,9 +537,109 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>03:45:20</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>04:53</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>68</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>03:45:20</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>05:17</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>92</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>03:45:20</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>05:22</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>97</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>03:45:20</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>05:44</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>119</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -569,7 +669,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:48:19</t>
+          <t>Última actualización: 03:45:20</t>
         </is>
       </c>
     </row>
@@ -604,7 +704,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:48:19</t>
+          <t>Última actualización: 03:45:20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1903
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-24.xlsx
+++ b/data/horarios-141-2026-03-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:45:20</t>
+          <t>Última actualización: 04:41:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>03:45:20</t>
+          <t>04:41:42</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>04:47</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>03:45:20</t>
+          <t>04:41:42</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>04:02</t>
+          <t>04:53</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>03:45:20</t>
+          <t>04:41:42</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04:48</t>
+          <t>05:16</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>63</v>
+        <v>35</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>03:45:20</t>
+          <t>04:41:42</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>04:53</t>
+          <t>05:22</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>68</v>
+        <v>41</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>03:45:20</t>
+          <t>04:41:42</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05:17</t>
+          <t>05:44</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>92</v>
+        <v>63</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>03:45:20</t>
+          <t>04:41:42</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>05:46</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>97</v>
+        <v>65</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,23 +623,173 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>03:45:20</t>
+          <t>04:41:42</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>05:44</t>
+          <t>06:01</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
+        <v>80</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>04:41:42</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06:09</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>88</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>04:41:42</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>91</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>04:41:42</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>109</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>04:41:42</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>06:34</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>113</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>04:41:42</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>06:39</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>118</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>04:41:42</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>06:40</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
         <v>119</v>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -656,7 +806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -669,14 +819,66 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:45:20</t>
+          <t>Última actualización: 04:41:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>04:41:42</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>91</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
         </is>
       </c>
     </row>
@@ -704,7 +906,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:45:20</t>
+          <t>Última actualización: 04:41:42</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1904
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-24.xlsx
+++ b/data/horarios-141-2026-03-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:41:42</t>
+          <t>Última actualización: 05:31:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:41:42</t>
+          <t>05:31:48</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>04:47</t>
+          <t>05:34</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04:41:42</t>
+          <t>05:31:48</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>04:53</t>
+          <t>05:46</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04:41:42</t>
+          <t>05:31:48</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05:16</t>
+          <t>06:09</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,17 +548,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04:41:42</t>
+          <t>05:31:48</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>06:12</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:41:42</t>
+          <t>05:31:48</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05:44</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04:41:42</t>
+          <t>05:31:48</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05:46</t>
+          <t>06:34</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>04:41:42</t>
+          <t>05:31:48</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:01</t>
+          <t>06:38</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>04:41:42</t>
+          <t>05:31:48</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:09</t>
+          <t>06:40</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>88</v>
+        <v>69</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,12 +673,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>04:41:42</t>
+          <t>05:31:48</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>06:55</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>04:41:42</t>
+          <t>05:31:48</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>109</v>
+        <v>88</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>04:41:42</t>
+          <t>05:31:48</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>06:34</t>
+          <t>07:19</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>04:41:42</t>
+          <t>05:31:48</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,23 +773,48 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>04:41:42</t>
+          <t>05:31:48</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>06:40</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
+        <v>115</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>05:31:48</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
         <v>119</v>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -806,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -819,14 +844,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:41:42</t>
+          <t>Última actualización: 05:31:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -860,7 +885,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:41:42</t>
+          <t>05:31:48</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -874,9 +899,59 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>91</v>
+        <v>41</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>05:31:48</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>06:55</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>84</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>05:31:48</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>07:19</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>108</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -906,7 +981,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:41:42</t>
+          <t>Última actualización: 05:31:48</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1905
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-24.xlsx
+++ b/data/horarios-141-2026-03-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:31:48</t>
+          <t>Última actualización: 06:32:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:31:48</t>
+          <t>06:32:38</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>05:34</t>
+          <t>06:33</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:31:48</t>
+          <t>06:32:38</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>05:46</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:31:48</t>
+          <t>06:32:38</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>06:09</t>
+          <t>06:40</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,12 +548,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>05:31:48</t>
+          <t>06:32:38</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>06:55</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05:31:48</t>
+          <t>06:32:38</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>05:31:48</t>
+          <t>06:32:38</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06:34</t>
+          <t>07:19</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05:31:48</t>
+          <t>06:32:38</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:38</t>
+          <t>07:19</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>67</v>
+        <v>47</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,12 +648,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05:31:48</t>
+          <t>06:32:38</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:40</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>69</v>
+        <v>48</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>05:31:48</t>
+          <t>06:32:38</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:55</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>84</v>
+        <v>54</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>05:31:48</t>
+          <t>06:32:38</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>06:59</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>88</v>
+        <v>55</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05:31:48</t>
+          <t>06:32:38</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>07:19</t>
+          <t>07:34</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>108</v>
+        <v>62</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>05:31:48</t>
+          <t>06:32:38</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>07:20</t>
+          <t>07:35</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>109</v>
+        <v>63</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>05:31:48</t>
+          <t>06:32:38</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>115</v>
+        <v>64</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,23 +798,98 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>05:31:48</t>
+          <t>06:32:38</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>08:09</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>119</v>
+        <v>97</v>
       </c>
       <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>06:32:38</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>08:17</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>105</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>06:32:38</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>08:21</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>109</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>06:32:38</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>08:28</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>116</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -844,7 +919,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:31:48</t>
+          <t>Última actualización: 06:32:38</t>
         </is>
       </c>
     </row>
@@ -885,12 +960,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:31:48</t>
+          <t>06:32:38</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>06:55</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -899,7 +974,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -910,21 +985,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:31:48</t>
+          <t>06:32:38</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>06:55</t>
+          <t>07:19</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>84</v>
+        <v>47</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -935,21 +1010,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:31:48</t>
+          <t>06:32:38</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>07:19</t>
+          <t>07:34</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>108</v>
+        <v>62</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -968,7 +1043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -981,14 +1056,66 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:31:48</t>
+          <t>Última actualización: 06:32:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>06:32:38</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>07:43</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>71</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1906
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-24.xlsx
+++ b/data/horarios-141-2026-03-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:32:38</t>
+          <t>Última actualización: 07:29:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 31</t>
         </is>
       </c>
     </row>
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>06:32:38</t>
+          <t>07:29:36</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>07:34</t>
+          <t>07:32</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>62</v>
+        <v>3</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>06:32:38</t>
+          <t>07:29:36</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>07:35</t>
+          <t>07:34</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>63</v>
+        <v>5</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -778,16 +778,16 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:35</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,21 +798,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>06:32:38</t>
+          <t>07:29:36</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>08:09</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>97</v>
+        <v>7</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,21 +823,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>06:32:38</t>
+          <t>07:29:36</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>08:17</t>
+          <t>07:55</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>105</v>
+        <v>26</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,21 +848,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>06:32:38</t>
+          <t>07:29:36</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>07:59</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>109</v>
+        <v>30</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,23 +873,373 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>07:29:36</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>08:01</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>32</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>06:32:38</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>08:09</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>97</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>07:29:36</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>08:17</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>48</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>07:29:36</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>08:21</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>52</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>07:29:36</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
         <is>
           <t>08:28</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D22" t="n">
-        <v>116</v>
-      </c>
-      <c r="E22" t="inlineStr">
+      <c r="D26" t="n">
+        <v>59</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>07:29:36</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>08:37</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>68</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>07:29:36</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>08:41</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>72</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>07:29:36</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>08:41</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>72</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>07:29:36</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>08:54</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>85</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>07:29:36</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>08:56</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>87</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>07:29:36</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>97</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>07:29:36</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>09:07</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>98</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>07:29:36</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>107</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>07:29:36</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>108</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>07:29:36</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>09:26</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>117</v>
+      </c>
+      <c r="E36" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -906,7 +1256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -919,14 +1269,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:32:38</t>
+          <t>Última actualización: 07:29:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -1010,7 +1360,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>06:32:38</t>
+          <t>07:29:36</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1024,9 +1374,84 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>62</v>
+        <v>5</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>07:29:36</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>08:37</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>68</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>07:29:36</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>08:54</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>85</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>07:29:36</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>08:56</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>87</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1043,7 +1468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1056,14 +1481,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:32:38</t>
+          <t>Última actualización: 07:29:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 4</t>
         </is>
       </c>
     </row>
@@ -1116,6 +1541,81 @@
       <c r="E6" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>07:29:36</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>07:44</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>15</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>07:29:36</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>08:33</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>64</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>07:29:36</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>08:47</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>78</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1907
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-24.xlsx
+++ b/data/horarios-141-2026-03-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:29:37</t>
+          <t>Última actualización: 08:24:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 31</t>
+          <t>Total filas: 45</t>
         </is>
       </c>
     </row>
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -973,7 +973,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>07:29:36</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>59</v>
+        <v>4</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1023,21 +1023,21 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>07:29:36</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>08:41</t>
+          <t>08:38</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>72</v>
+        <v>14</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1048,7 +1048,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>07:29:36</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1062,7 +1062,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>72</v>
+        <v>17</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1073,21 +1073,21 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>07:29:36</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>08:54</t>
+          <t>08:41</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>85</v>
+        <v>17</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,21 +1098,21 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>07:29:36</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>08:56</t>
+          <t>08:49</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>87</v>
+        <v>25</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,21 +1123,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>07:29:36</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>08:54</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>97</v>
+        <v>30</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1153,16 +1153,16 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>09:07</t>
+          <t>08:56</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,21 +1173,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>07:29:36</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>08:57</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>107</v>
+        <v>33</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,21 +1198,21 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>07:29:36</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>108</v>
+        <v>42</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1228,18 +1228,368 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
+          <t>09:07</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>98</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>09:11</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>47</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>07:29:36</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>107</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>53</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>53</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>07:29:36</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
           <t>09:26</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D36" t="n">
+      <c r="D41" t="n">
         <v>117</v>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>09:27</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>63</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>09:38</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>74</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>09:42</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>78</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>09:43</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>79</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>09:52</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>88</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>09:56</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>92</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>09:58</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>94</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>106</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>10:13</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>109</v>
+      </c>
+      <c r="E50" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1256,7 +1606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1269,14 +1619,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:29:37</t>
+          <t>Última actualización: 08:24:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 6</t>
+          <t>Total filas: 9</t>
         </is>
       </c>
     </row>
@@ -1410,21 +1760,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07:29:36</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>08:54</t>
+          <t>08:38</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>85</v>
+        <v>14</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1435,23 +1785,98 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>08:54</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>30</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>07:29:36</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>08:56</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="D12" t="n">
         <v>87</v>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>08:57</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>33</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>09:58</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>94</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1468,7 +1893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1481,14 +1906,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:29:37</t>
+          <t>Última actualización: 08:24:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -1572,7 +1997,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>07:29:36</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1586,7 +2011,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>64</v>
+        <v>9</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1614,6 +2039,81 @@
         <v>78</v>
       </c>
       <c r="E9" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>08:48</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>24</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>09:28</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>64</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>08:24:08</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>10:08</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>104</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1908
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-24.xlsx
+++ b/data/horarios-141-2026-03-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:24:08</t>
+          <t>Última actualización: 09:00:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 45</t>
+          <t>Total filas: 56</t>
         </is>
       </c>
     </row>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>09:00:34</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>42</v>
+        <v>6</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>09:00:34</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1258,11 +1258,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>47</v>
+        <v>11</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,21 +1273,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>07:29:36</t>
+          <t>09:00:34</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>107</v>
+        <v>11</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,12 +1298,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>09:00:34</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1312,7 +1312,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>53</v>
+        <v>16</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1348,21 +1348,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>07:29:36</t>
+          <t>09:00:34</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>09:26</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>117</v>
+        <v>17</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,21 +1373,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>09:00:34</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>09:27</t>
+          <t>09:25</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>63</v>
+        <v>25</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,21 +1398,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>09:00:34</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>09:38</t>
+          <t>09:26</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>74</v>
+        <v>26</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1428,16 +1428,16 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>09:42</t>
+          <t>09:27</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,21 +1448,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>09:00:34</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>09:43</t>
+          <t>09:38</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>79</v>
+        <v>38</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,21 +1473,21 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>09:00:34</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>09:52</t>
+          <t>09:41</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>88</v>
+        <v>41</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1503,16 +1503,16 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>09:56</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,21 +1523,21 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>09:00:34</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>09:58</t>
+          <t>09:43</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>94</v>
+        <v>43</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1553,16 +1553,16 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>10:10</t>
+          <t>09:52</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>106</v>
+        <v>88</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,23 +1573,298 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t>09:00:34</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>55</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>09:00:34</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>09:56</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>56</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>09:00:34</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>09:58</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>58</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
           <t>08:24:08</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>106</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>09:00:34</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>10:11</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>71</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>09:00:34</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
         <is>
           <t>10:13</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C55" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D50" t="n">
-        <v>109</v>
-      </c>
-      <c r="E50" t="inlineStr">
+      <c r="D55" t="n">
+        <v>73</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>09:00:34</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>10:26</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>86</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>09:00:34</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>10:27</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>87</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>09:00:34</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>15_P INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>103</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>09:00:34</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>104</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>09:00:34</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>10:56</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>116</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>09:00:34</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>10:58</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>118</v>
+      </c>
+      <c r="E61" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1619,7 +1894,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:24:08</t>
+          <t>Última actualización: 09:00:34</t>
         </is>
       </c>
     </row>
@@ -1860,7 +2135,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>09:00:34</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1874,7 +2149,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>94</v>
+        <v>58</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1893,7 +2168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1906,14 +2181,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:24:08</t>
+          <t>Última actualización: 09:00:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -2072,7 +2347,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>09:00:34</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2086,7 +2361,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -2097,25 +2372,100 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>09:00:34</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>10:07</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>67</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>08:24:08</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>10:08</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D13" t="n">
         <v>104</v>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>09:00:34</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>10:28</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>88</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>09:00:34</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>10:35</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>95</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1909
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-24.xlsx
+++ b/data/horarios-141-2026-03-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:00:34</t>
+          <t>Última actualización: 10:45:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 56</t>
+          <t>Total filas: 77</t>
         </is>
       </c>
     </row>
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>09:00:34</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>09:00:34</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1823,21 +1823,21 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>09:00:34</t>
+          <t>10:45:13</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>10:56</t>
+          <t>10:45</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>116</v>
+        <v>0</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,23 +1848,548 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
+          <t>10:45:13</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>10</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>10:45:13</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>10</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
           <t>09:00:34</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>10:56</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>116</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>10:45:13</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>10:57</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>12</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>10:45:13</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
         <is>
           <t>10:58</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C65" t="inlineStr">
         <is>
           <t>81_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D61" t="n">
-        <v>118</v>
-      </c>
-      <c r="E61" t="inlineStr">
+      <c r="D65" t="n">
+        <v>13</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>10:45:13</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>11:03</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>18</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>10:45:13</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>11:10</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>25</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>10:45:13</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>11:10</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>25</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>10:45:13</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>11:13</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>28</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>10:45:13</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>35</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>10:45:13</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>11:25</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>40</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>10:45:13</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>11:28</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>43</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>10:45:13</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>11:39</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>54</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>10:45:13</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>11:42</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>57</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>10:45:13</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>11:53</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>68</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>10:45:13</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>11:58</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>73</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>10:45:13</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>12:09</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>84</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>10:45:13</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>12:13</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>88</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>10:45:13</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>12:28</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>103</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>10:45:13</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>12:37</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>112</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>10:45:13</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>12:39</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>114</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>10:45:13</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>12:42</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>117</v>
+      </c>
+      <c r="E82" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1881,7 +2406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1894,14 +2419,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:00:34</t>
+          <t>Última actualización: 10:45:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 9</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -2152,6 +2677,81 @@
         <v>58</v>
       </c>
       <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>10:45:13</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>11:28</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>43</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>10:45:13</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>11:39</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>54</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>10:45:13</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>12:28</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>103</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2168,7 +2768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2181,14 +2781,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:00:34</t>
+          <t>Última actualización: 10:45:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 11</t>
         </is>
       </c>
     </row>
@@ -2466,6 +3066,31 @@
       <c r="E15" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>10:45:13</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>11:28</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>43</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1910
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-24.xlsx
+++ b/data/horarios-141-2026-03-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E82"/>
+  <dimension ref="A1:E95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:45:13</t>
+          <t>Última actualización: 11:44:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 77</t>
+          <t>Total filas: 90</t>
         </is>
       </c>
     </row>
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>09:00:34</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>09:00:34</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -2198,21 +2198,21 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>10:45:13</t>
+          <t>11:44:14</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>11:53</t>
+          <t>11:45</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>68</v>
+        <v>1</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2223,21 +2223,21 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>10:45:13</t>
+          <t>11:44:14</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>11:58</t>
+          <t>11:53</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>73</v>
+        <v>9</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,21 +2248,21 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>10:45:13</t>
+          <t>11:44:14</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>12:09</t>
+          <t>11:55</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>84</v>
+        <v>11</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,21 +2273,21 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>10:45:13</t>
+          <t>11:44:14</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>12:13</t>
+          <t>11:58</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>88</v>
+        <v>14</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2298,21 +2298,21 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>10:45:13</t>
+          <t>11:44:14</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>12:28</t>
+          <t>12:09</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>103</v>
+        <v>25</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2323,21 +2323,21 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>10:45:13</t>
+          <t>11:44:14</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>12:37</t>
+          <t>12:09</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>112</v>
+        <v>25</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,21 +2348,21 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>10:45:13</t>
+          <t>11:44:14</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>12:39</t>
+          <t>12:10</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>114</v>
+        <v>26</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,23 +2373,348 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>10:45:13</t>
+          <t>11:44:14</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
+          <t>12:13</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>29</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>11:44:14</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>12:23</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>39</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>11:44:14</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>12:28</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>44</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>11:44:14</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>12:37</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>53</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>11:44:14</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>12:39</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>55</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>11:44:14</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>12:41</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>57</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>11:44:14</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
           <t>12:42</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr">
+      <c r="C88" t="inlineStr">
         <is>
           <t>15X38_ABASTO</t>
         </is>
       </c>
-      <c r="D82" t="n">
-        <v>117</v>
-      </c>
-      <c r="E82" t="inlineStr">
+      <c r="D88" t="n">
+        <v>58</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>11:44:14</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>12:57</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>73</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>11:44:14</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>12:58</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>74</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>11:44:14</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>13:13</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>89</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>11:44:14</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>13:14</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>90</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>11:44:14</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>100</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>11:44:14</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>13:33</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>109</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>11:44:14</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>13:40</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>116</v>
+      </c>
+      <c r="E95" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2406,7 +2731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2419,14 +2744,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:45:13</t>
+          <t>Última actualización: 11:44:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -2735,23 +3060,98 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>10:45:13</t>
+          <t>11:44:14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>11:44:14</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
           <t>12:28</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D17" t="n">
-        <v>103</v>
-      </c>
-      <c r="E17" t="inlineStr">
+      <c r="D18" t="n">
+        <v>44</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>11:44:14</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>12:58</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>74</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>11:44:14</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>100</v>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2768,7 +3168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2781,14 +3181,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:45:13</t>
+          <t>Última actualización: 11:44:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 11</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -3091,6 +3491,56 @@
       <c r="E16" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>11:44:14</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>12:58</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>74</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>11:44:14</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>13:29</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>105</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1911
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-24.xlsx
+++ b/data/horarios-141-2026-03-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E95"/>
+  <dimension ref="A1:E113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:44:14</t>
+          <t>Última actualización: 12:46:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 90</t>
+          <t>Total filas: 108</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>09:00:34</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>09:00:34</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -2548,21 +2548,21 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>11:44:14</t>
+          <t>12:46:57</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>73</v>
+        <v>9</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2573,21 +2573,21 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>11:44:14</t>
+          <t>12:46:57</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>12:58</t>
+          <t>12:56</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>74</v>
+        <v>10</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2603,16 +2603,16 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>13:13</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,21 +2623,21 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>11:44:14</t>
+          <t>12:46:57</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>13:14</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>90</v>
+        <v>11</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2653,16 +2653,16 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>12:58</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>100</v>
+        <v>74</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2673,21 +2673,21 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>11:44:14</t>
+          <t>12:46:57</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>13:33</t>
+          <t>13:12</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>109</v>
+        <v>26</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2703,18 +2703,468 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
+          <t>13:13</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>89</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>12:46:57</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>13:13</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>27</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>11:44:14</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>13:14</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>90</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>12:46:57</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>13:21</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>35</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>12:46:57</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>38</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>12:46:57</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>39</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>12:46:57</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>46</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>11:44:14</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>13:33</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>109</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>12:46:57</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>13:39</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>53</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>11:44:14</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
           <t>13:40</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr">
+      <c r="C104" t="inlineStr">
         <is>
           <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
-      <c r="D95" t="n">
+      <c r="D104" t="n">
         <v>116</v>
       </c>
-      <c r="E95" t="inlineStr">
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>12:46:57</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>13:46</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>60</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>12:46:57</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>13:49</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>63</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>12:46:57</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>14:07</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>81</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>12:46:57</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>14:07</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>81</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>12:46:57</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>14:11</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>85</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>12:46:57</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>90</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>12:46:57</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>14:26</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>100</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>12:46:57</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>14:27</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>101</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>12:46:57</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>114</v>
+      </c>
+      <c r="E113" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2731,7 +3181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2744,14 +3194,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:44:14</t>
+          <t>Última actualización: 12:46:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -3110,12 +3560,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>11:44:14</t>
+          <t>12:46:57</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>12:58</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -3124,7 +3574,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>74</v>
+        <v>11</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -3140,18 +3590,68 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
+          <t>12:58</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>74</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>12:46:57</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
           <t>13:24</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D20" t="n">
-        <v>100</v>
-      </c>
-      <c r="E20" t="inlineStr">
+      <c r="D21" t="n">
+        <v>38</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>12:46:57</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>14:27</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>101</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3168,7 +3668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3181,14 +3681,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:44:14</t>
+          <t>Última actualización: 12:46:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -3497,12 +3997,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>11:44:14</t>
+          <t>12:46:57</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>12:58</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -3511,7 +4011,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>74</v>
+        <v>11</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -3527,20 +4027,95 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>12:58</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>74</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>12:46:57</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>13:28</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>42</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>11:44:14</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
           <t>13:29</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D18" t="n">
+      <c r="D20" t="n">
         <v>105</v>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>12:46:57</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>13:52</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>66</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1912
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-24.xlsx
+++ b/data/horarios-141-2026-03-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E113"/>
+  <dimension ref="A1:E126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:46:57</t>
+          <t>Última actualización: 13:42:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 108</t>
+          <t>Total filas: 121</t>
         </is>
       </c>
     </row>
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>09:00:34</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>09:00:34</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -2008,7 +2008,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -2033,7 +2033,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>11:44:14</t>
+          <t>12:46:57</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>89</v>
+        <v>27</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>12:46:57</t>
+          <t>11:44:14</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>27</v>
+        <v>89</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2973,21 +2973,21 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>12:46:57</t>
+          <t>13:42:53</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>13:49</t>
+          <t>13:47</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>63</v>
+        <v>5</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,21 +2998,21 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>12:46:57</t>
+          <t>13:42:53</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>14:07</t>
+          <t>13:49</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>81</v>
+        <v>7</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,21 +3023,21 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>12:46:57</t>
+          <t>13:42:53</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>14:07</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>81</v>
+        <v>13</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3053,16 +3053,16 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>14:11</t>
+          <t>14:07</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,21 +3073,21 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>12:46:57</t>
+          <t>13:42:53</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:07</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>90</v>
+        <v>25</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3098,21 +3098,21 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>12:46:57</t>
+          <t>13:42:53</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>14:26</t>
+          <t>14:08</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>100</v>
+        <v>26</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,21 +3123,21 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>12:46:57</t>
+          <t>13:42:53</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>14:27</t>
+          <t>14:11</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>101</v>
+        <v>29</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3148,23 +3148,348 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>12:46:57</t>
+          <t>13:42:53</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>34</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>13:42:53</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>43</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>13:42:53</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>14:26</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>44</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>13:42:53</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>14:27</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>45</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>13:42:53</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
           <t>14:40</t>
         </is>
       </c>
-      <c r="C113" t="inlineStr">
+      <c r="C117" t="inlineStr">
         <is>
           <t>14X44_ABASTO</t>
         </is>
       </c>
-      <c r="D113" t="n">
-        <v>114</v>
-      </c>
-      <c r="E113" t="inlineStr">
+      <c r="D117" t="n">
+        <v>58</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>13:42:53</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>14:47</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>65</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>13:42:53</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>14:56</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>74</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>13:42:53</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>14:59</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>77</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>13:42:53</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>15:07</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>85</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>13:42:53</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>88</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>13:42:53</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>88</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>13:42:53</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>15:26</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>104</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>13:42:53</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>15:27</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>105</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>13:42:53</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>15:38</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>116</v>
+      </c>
+      <c r="E126" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3181,7 +3506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3194,14 +3519,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:46:57</t>
+          <t>Última actualización: 13:42:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 20</t>
         </is>
       </c>
     </row>
@@ -3635,7 +3960,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12:46:57</t>
+          <t>13:42:53</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3649,9 +3974,84 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>101</v>
+        <v>45</v>
       </c>
       <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>13:42:53</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>14:47</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>65</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>13:42:53</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>14:56</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>74</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>13:42:53</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>15:27</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>105</v>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3668,7 +4068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3681,14 +4081,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:46:57</t>
+          <t>Última actualización: 13:42:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -4097,7 +4497,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12:46:57</t>
+          <t>13:42:53</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -4111,11 +4511,61 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>66</v>
+        <v>10</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>13:42:53</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>14:27</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>45</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>13:42:53</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>15:12</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>90</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1913
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-24.xlsx
+++ b/data/horarios-141-2026-03-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E126"/>
+  <dimension ref="A1:E142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:42:53</t>
+          <t>Última actualización: 14:39:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 121</t>
+          <t>Total filas: 137</t>
         </is>
       </c>
     </row>
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>12:46:57</t>
+          <t>11:44:14</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>27</v>
+        <v>89</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>11:44:14</t>
+          <t>12:46:57</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>89</v>
+        <v>27</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>12:46:57</t>
+          <t>13:42:53</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>81</v>
+        <v>25</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>13:42:53</t>
+          <t>12:46:57</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>25</v>
+        <v>81</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3273,21 +3273,21 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>13:42:53</t>
+          <t>14:39:41</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>14:47</t>
+          <t>14:41</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>65</v>
+        <v>2</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3303,16 +3303,16 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>14:56</t>
+          <t>14:47</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,21 +3323,21 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>13:42:53</t>
+          <t>14:39:41</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:48</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>77</v>
+        <v>9</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,21 +3348,21 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>13:42:53</t>
+          <t>14:39:41</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>15:07</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>85</v>
+        <v>16</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,21 +3373,21 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>13:42:53</t>
+          <t>14:39:41</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>15:10</t>
+          <t>14:56</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>88</v>
+        <v>17</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3403,16 +3403,16 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>15:10</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,21 +3423,21 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>13:42:53</t>
+          <t>14:39:41</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>15:26</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>104</v>
+        <v>22</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,21 +3448,21 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>13:42:53</t>
+          <t>14:39:41</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>15:27</t>
+          <t>15:07</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>105</v>
+        <v>28</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3478,18 +3478,418 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>88</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>14:39:41</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>31</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>14:39:41</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>15:11</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>32</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>14:39:41</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>15:25</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>46</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>14:39:41</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>15:26</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>47</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>14:39:41</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>15:27</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>48</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>13:42:53</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
           <t>15:38</t>
         </is>
       </c>
-      <c r="C126" t="inlineStr">
+      <c r="C132" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D126" t="n">
+      <c r="D132" t="n">
         <v>116</v>
       </c>
-      <c r="E126" t="inlineStr">
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>14:39:41</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>15:41</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>62</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>14:39:41</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>15:48</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>69</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>14:39:41</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>15:52</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>73</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>14:39:41</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>77</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>14:39:41</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>16:01</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>82</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>14:39:41</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>16:07</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>88</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>14:39:41</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>16:08</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>89</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>14:39:41</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>16:23</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>104</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>14:39:41</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>16:26</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>107</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>14:39:41</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>16:38</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>119</v>
+      </c>
+      <c r="E142" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3506,7 +3906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3519,14 +3919,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:42:53</t>
+          <t>Última actualización: 14:39:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 20</t>
+          <t>Total filas: 21</t>
         </is>
       </c>
     </row>
@@ -4010,21 +4410,21 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>13:42:53</t>
+          <t>14:39:41</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>14:56</t>
+          <t>14:48</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>74</v>
+        <v>9</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -4035,23 +4435,48 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>13:42:53</t>
+          <t>14:39:41</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>14:56</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>17</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>14:39:41</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
           <t>15:27</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D25" t="n">
-        <v>105</v>
-      </c>
-      <c r="E25" t="inlineStr">
+      <c r="D26" t="n">
+        <v>48</v>
+      </c>
+      <c r="E26" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4068,7 +4493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4081,14 +4506,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:42:53</t>
+          <t>Última actualización: 14:39:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 20</t>
         </is>
       </c>
     </row>
@@ -4547,7 +4972,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>13:42:53</t>
+          <t>14:39:41</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -4561,9 +4986,59 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>90</v>
+        <v>33</v>
       </c>
       <c r="E23" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>14:39:41</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>15:52</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>73</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>14:39:41</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>16:37</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>118</v>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1914
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-24.xlsx
+++ b/data/horarios-141-2026-03-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E142"/>
+  <dimension ref="A1:E155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:39:41</t>
+          <t>Última actualización: 15:36:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 137</t>
+          <t>Total filas: 150</t>
         </is>
       </c>
     </row>
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>11:44:14</t>
+          <t>12:46:57</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>73</v>
+        <v>11</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>12:46:57</t>
+          <t>11:44:14</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2633,11 +2633,11 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>11</v>
+        <v>73</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>11:44:14</t>
+          <t>12:46:57</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>89</v>
+        <v>27</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>12:46:57</t>
+          <t>11:44:14</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>27</v>
+        <v>89</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>13:42:53</t>
+          <t>12:46:57</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>25</v>
+        <v>81</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>12:46:57</t>
+          <t>13:42:53</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>81</v>
+        <v>25</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>14:39:41</t>
+          <t>15:36:41</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3662,7 +3662,7 @@
         </is>
       </c>
       <c r="D133" t="n">
-        <v>62</v>
+        <v>5</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,7 +3673,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>14:39:41</t>
+          <t>15:36:41</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -3687,7 +3687,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>69</v>
+        <v>12</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,21 +3698,21 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>14:39:41</t>
+          <t>15:36:41</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>15:52</t>
+          <t>15:51</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>73</v>
+        <v>15</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3728,16 +3728,16 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:52</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,21 +3748,21 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>14:39:41</t>
+          <t>15:36:41</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>16:01</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>82</v>
+        <v>19</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,21 +3773,21 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>14:39:41</t>
+          <t>15:36:41</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>16:07</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>88</v>
+        <v>20</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3798,21 +3798,21 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>14:39:41</t>
+          <t>15:36:41</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>16:08</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>89</v>
+        <v>20</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3828,16 +3828,16 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>16:01</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>104</v>
+        <v>82</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3848,21 +3848,21 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>14:39:41</t>
+          <t>15:36:41</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>16:26</t>
+          <t>16:07</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>107</v>
+        <v>31</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3878,18 +3878,343 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
+          <t>16:08</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>89</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>15:36:41</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>16:11</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>35</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>15:36:41</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>16:23</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>47</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>15:36:41</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>16:25</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>49</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>15:36:41</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>16:26</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>50</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>15:36:41</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
           <t>16:38</t>
         </is>
       </c>
-      <c r="C142" t="inlineStr">
+      <c r="C147" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D142" t="n">
-        <v>119</v>
-      </c>
-      <c r="E142" t="inlineStr">
+      <c r="D147" t="n">
+        <v>62</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>15:36:41</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>16:40</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>64</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>15:36:41</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>16:41</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>65</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>15:36:41</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>16:53</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>77</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>15:36:41</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>16:56</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>80</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>15:36:41</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>17:07</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>91</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>15:36:41</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>17:22</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>106</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>15:36:41</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>17:31</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>115</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>15:36:41</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>17:32</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>116</v>
+      </c>
+      <c r="E155" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3906,7 +4231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3919,14 +4244,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:39:41</t>
+          <t>Última actualización: 15:36:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 21</t>
+          <t>Total filas: 23</t>
         </is>
       </c>
     </row>
@@ -4477,6 +4802,56 @@
         <v>48</v>
       </c>
       <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>15:36:41</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>17:07</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>91</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>15:36:41</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>17:32</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>116</v>
+      </c>
+      <c r="E28" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4493,7 +4868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4506,14 +4881,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:39:41</t>
+          <t>Última actualización: 15:36:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 20</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -4997,7 +5372,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>14:39:41</t>
+          <t>15:36:41</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -5011,7 +5386,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>73</v>
+        <v>16</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -5041,6 +5416,56 @@
       <c r="E25" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>15:36:41</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>16:38</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>62</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>15:36:41</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>17:02</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>86</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1915
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-24.xlsx
+++ b/data/horarios-141-2026-03-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E155"/>
+  <dimension ref="A1:E169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:36:41</t>
+          <t>Última actualización: 16:36:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 150</t>
+          <t>Total filas: 164</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -3783,7 +3783,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -3998,7 +3998,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>15:36:41</t>
+          <t>16:36:44</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4012,7 +4012,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>62</v>
+        <v>2</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>15:36:41</t>
+          <t>16:36:44</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4037,7 +4037,7 @@
         </is>
       </c>
       <c r="D148" t="n">
-        <v>64</v>
+        <v>4</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,7 +4048,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>15:36:41</t>
+          <t>16:36:44</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -4062,7 +4062,7 @@
         </is>
       </c>
       <c r="D149" t="n">
-        <v>65</v>
+        <v>5</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,21 +4073,21 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>15:36:41</t>
+          <t>16:36:44</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>16:53</t>
+          <t>16:41</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>77</v>
+        <v>5</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,21 +4098,21 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>15:36:41</t>
+          <t>16:36:44</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>16:56</t>
+          <t>16:53</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>80</v>
+        <v>17</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,21 +4123,21 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>15:36:41</t>
+          <t>16:36:44</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>17:07</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>91</v>
+        <v>19</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,21 +4148,21 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>15:36:41</t>
+          <t>16:36:44</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>17:22</t>
+          <t>16:56</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>106</v>
+        <v>20</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,21 +4173,21 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>15:36:41</t>
+          <t>16:36:44</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>17:31</t>
+          <t>17:07</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>115</v>
+        <v>31</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,23 +4198,373 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
+          <t>16:36:44</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>17:22</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>46</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>16:36:44</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>17:25</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>49</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
           <t>15:36:41</t>
         </is>
       </c>
-      <c r="B155" t="inlineStr">
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>17:31</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>115</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>16:36:44</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
         <is>
           <t>17:32</t>
         </is>
       </c>
-      <c r="C155" t="inlineStr">
+      <c r="C158" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D155" t="n">
-        <v>116</v>
-      </c>
-      <c r="E155" t="inlineStr">
+      <c r="D158" t="n">
+        <v>56</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>16:36:44</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>60</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>16:36:44</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>17:38</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>62</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>16:36:44</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>17:38</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>62</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>16:36:44</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>17:50</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>74</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>16:36:44</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>17:52</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>76</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>16:36:44</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>18:05</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>89</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>16:36:44</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>92</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>16:36:44</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>18:10</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>94</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>16:36:44</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>104</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>16:36:44</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>18:22</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>106</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>16:36:44</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>18:35</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>119</v>
+      </c>
+      <c r="E169" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4231,7 +4581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4244,14 +4594,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:36:41</t>
+          <t>Última actualización: 16:36:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 23</t>
+          <t>Total filas: 25</t>
         </is>
       </c>
     </row>
@@ -4810,7 +5160,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>15:36:41</t>
+          <t>16:36:44</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -4824,7 +5174,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>91</v>
+        <v>31</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -4835,7 +5185,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>15:36:41</t>
+          <t>16:36:44</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -4849,9 +5199,59 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>116</v>
+        <v>56</v>
       </c>
       <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>16:36:44</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>17:52</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>76</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>16:36:44</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>18:22</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>106</v>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4868,7 +5268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4881,14 +5281,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:36:41</t>
+          <t>Última actualización: 16:36:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 23</t>
         </is>
       </c>
     </row>
@@ -5397,7 +5797,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>14:39:41</t>
+          <t>16:36:44</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -5411,7 +5811,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>118</v>
+        <v>1</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -5447,7 +5847,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>15:36:41</t>
+          <t>16:36:44</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -5461,9 +5861,34 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>86</v>
+        <v>26</v>
       </c>
       <c r="E27" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>16:36:44</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>18:29</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>113</v>
+      </c>
+      <c r="E28" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1916
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-24.xlsx
+++ b/data/horarios-141-2026-03-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E169"/>
+  <dimension ref="A1:E180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:36:44</t>
+          <t>Última actualización: 17:05:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 164</t>
+          <t>Total filas: 175</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>09:00:34</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>09:00:34</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -2008,7 +2008,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -2033,7 +2033,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -4058,7 +4058,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -4083,7 +4083,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -4198,21 +4198,21 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>16:36:44</t>
+          <t>17:05:08</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>17:22</t>
+          <t>17:08</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>46</v>
+        <v>3</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,21 +4223,21 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>16:36:44</t>
+          <t>17:05:08</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>17:25</t>
+          <t>17:22</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4248,21 +4248,21 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>15:36:41</t>
+          <t>17:05:08</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>17:31</t>
+          <t>17:25</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>115</v>
+        <v>20</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,21 +4273,21 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>16:36:44</t>
+          <t>17:05:08</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>17:32</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>56</v>
+        <v>26</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4303,16 +4303,16 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,21 +4323,21 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>16:36:44</t>
+          <t>17:05:08</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>17:38</t>
+          <t>17:33</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>62</v>
+        <v>28</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4353,16 +4353,16 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>17:38</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,21 +4373,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>16:36:44</t>
+          <t>17:05:08</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>17:50</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>74</v>
+        <v>32</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,21 +4398,21 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>16:36:44</t>
+          <t>17:05:08</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>17:52</t>
+          <t>17:38</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4428,16 +4428,16 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>17:38</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>89</v>
+        <v>62</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,21 +4448,21 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>16:36:44</t>
+          <t>17:05:08</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>18:08</t>
+          <t>17:50</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>92</v>
+        <v>45</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4478,16 +4478,16 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>17:52</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,21 +4498,21 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>16:36:44</t>
+          <t>17:05:08</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>17:53</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>104</v>
+        <v>48</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4528,16 +4528,16 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>18:22</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>106</v>
+        <v>89</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,23 +4548,298 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
+          <t>17:05:08</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>18:06</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>61</v>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>17:05:08</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>63</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>17:05:08</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>18:10</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>65</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>17:05:08</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>18:19</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>74</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>17:05:08</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>75</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
           <t>16:36:44</t>
         </is>
       </c>
-      <c r="B169" t="inlineStr">
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>18:22</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>106</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>17:05:08</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>78</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>17:05:08</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>79</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>16:36:44</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
         <is>
           <t>18:35</t>
         </is>
       </c>
-      <c r="C169" t="inlineStr">
+      <c r="C177" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D169" t="n">
+      <c r="D177" t="n">
         <v>119</v>
       </c>
-      <c r="E169" t="inlineStr">
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>17:05:08</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>91</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>17:05:08</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>18:37</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>92</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>17:05:08</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>18:53</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>108</v>
+      </c>
+      <c r="E180" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4581,7 +4856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4594,14 +4869,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:36:44</t>
+          <t>Última actualización: 17:05:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 25</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -5185,21 +5460,21 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>16:36:44</t>
+          <t>17:05:08</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>17:32</t>
+          <t>17:08</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>56</v>
+        <v>3</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -5215,16 +5490,16 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>17:52</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>76</v>
+        <v>56</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -5235,23 +5510,123 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>17:05:08</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>17:33</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>28</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>16:36:44</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>17:52</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>76</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>17:05:08</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>17:53</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>48</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>16:36:44</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
         <is>
           <t>18:22</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D30" t="n">
+      <c r="D33" t="n">
         <v>106</v>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>17:05:08</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>78</v>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5268,7 +5643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5281,14 +5656,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:36:44</t>
+          <t>Última actualización: 17:05:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 23</t>
+          <t>Total filas: 25</t>
         </is>
       </c>
     </row>
@@ -5891,6 +6266,56 @@
       <c r="E28" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>17:05:08</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>85</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>17:05:08</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>19:02</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>117</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1917
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-24.xlsx
+++ b/data/horarios-141-2026-03-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E180"/>
+  <dimension ref="A1:E193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:05:08</t>
+          <t>Última actualización: 17:53:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 175</t>
+          <t>Total filas: 188</t>
         </is>
       </c>
     </row>
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -2008,7 +2008,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -2033,7 +2033,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>12:46:57</t>
+          <t>11:44:14</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>27</v>
+        <v>89</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>11:44:14</t>
+          <t>12:46:57</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>89</v>
+        <v>27</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -4058,7 +4058,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -4083,7 +4083,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -4498,7 +4498,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>17:05:08</t>
+          <t>17:53:42</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4512,7 +4512,7 @@
         </is>
       </c>
       <c r="D167" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,7 +4523,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>16:36:44</t>
+          <t>17:53:42</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -4537,7 +4537,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>89</v>
+        <v>12</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4573,7 +4573,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>17:05:08</t>
+          <t>17:53:42</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -4587,7 +4587,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>63</v>
+        <v>15</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>17:05:08</t>
+          <t>17:53:42</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4612,7 +4612,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>65</v>
+        <v>17</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4648,7 +4648,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>17:05:08</t>
+          <t>17:53:42</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -4662,7 +4662,7 @@
         </is>
       </c>
       <c r="D173" t="n">
-        <v>75</v>
+        <v>27</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,21 +4673,21 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>16:36:44</t>
+          <t>17:53:42</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>18:22</t>
+          <t>18:21</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>106</v>
+        <v>28</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,12 +4698,12 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>17:05:08</t>
+          <t>17:53:42</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:22</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -4712,7 +4712,7 @@
         </is>
       </c>
       <c r="D175" t="n">
-        <v>78</v>
+        <v>29</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4728,16 +4728,16 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,21 +4748,21 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>16:36:44</t>
+          <t>17:05:08</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>119</v>
+        <v>79</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,21 +4773,21 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>17:05:08</t>
+          <t>17:53:42</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>91</v>
+        <v>32</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,21 +4798,21 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>17:05:08</t>
+          <t>17:53:42</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>18:37</t>
+          <t>18:35</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>92</v>
+        <v>42</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4828,18 +4828,343 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>91</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>17:53:42</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>18:37</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>44</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>17:53:42</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>18:50</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>57</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>17:53:42</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
           <t>18:53</t>
         </is>
       </c>
-      <c r="C180" t="inlineStr">
+      <c r="C183" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D180" t="n">
-        <v>108</v>
-      </c>
-      <c r="E180" t="inlineStr">
+      <c r="D183" t="n">
+        <v>60</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>17:53:42</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>18:55</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>62</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>17:53:42</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>19:05</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>72</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>17:53:42</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>19:07</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>74</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>17:53:42</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>19:14</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>81</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>17:53:42</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>19:17</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>84</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>17:53:42</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>19:21</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>88</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>17:53:42</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>19:22</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>89</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>17:53:42</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>19:33</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>100</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>17:53:42</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>107</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>17:53:42</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>19:43</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>110</v>
+      </c>
+      <c r="E193" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4856,7 +5181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4869,14 +5194,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:05:08</t>
+          <t>Última actualización: 17:53:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 31</t>
         </is>
       </c>
     </row>
@@ -5560,7 +5885,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>17:05:08</t>
+          <t>17:53:42</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5574,7 +5899,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -5585,7 +5910,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>16:36:44</t>
+          <t>17:53:42</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -5599,7 +5924,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>106</v>
+        <v>29</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -5627,6 +5952,56 @@
         <v>78</v>
       </c>
       <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>17:53:42</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>19:07</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>74</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>17:53:42</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>19:22</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>89</v>
+      </c>
+      <c r="E36" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5643,7 +6018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5656,14 +6031,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:05:08</t>
+          <t>Última actualización: 17:53:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 25</t>
+          <t>Total filas: 27</t>
         </is>
       </c>
     </row>
@@ -6297,23 +6672,73 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>17:53:42</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>18:41</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>48</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>17:53:42</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>19:01</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>68</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>17:05:08</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>19:02</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D30" t="n">
+      <c r="D32" t="n">
         <v>117</v>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1918
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-24.xlsx
+++ b/data/horarios-141-2026-03-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E193"/>
+  <dimension ref="A1:E205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:53:42</t>
+          <t>Última actualización: 18:27:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 188</t>
+          <t>Total filas: 200</t>
         </is>
       </c>
     </row>
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>11:44:14</t>
+          <t>12:46:57</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>89</v>
+        <v>27</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>12:46:57</t>
+          <t>11:44:14</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>27</v>
+        <v>89</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>12:46:57</t>
+          <t>13:42:53</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>81</v>
+        <v>25</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>13:42:53</t>
+          <t>12:46:57</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>25</v>
+        <v>81</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -4058,7 +4058,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -4083,7 +4083,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -4798,7 +4798,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>17:53:42</t>
+          <t>18:27:26</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -4812,7 +4812,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>17:53:42</t>
+          <t>18:27:26</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4862,7 +4862,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>44</v>
+        <v>10</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4873,7 +4873,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>17:53:42</t>
+          <t>18:27:26</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -4887,7 +4887,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>57</v>
+        <v>23</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>17:53:42</t>
+          <t>18:27:26</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4912,7 +4912,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>60</v>
+        <v>26</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>17:53:42</t>
+          <t>18:27:26</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4962,7 +4962,7 @@
         </is>
       </c>
       <c r="D185" t="n">
-        <v>72</v>
+        <v>38</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4998,21 +4998,21 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>17:53:42</t>
+          <t>18:27:26</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>19:14</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>81</v>
+        <v>41</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5028,16 +5028,16 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:14</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5053,16 +5053,16 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,21 +5073,21 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>17:53:42</t>
+          <t>18:27:26</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>19:22</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>89</v>
+        <v>50</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,21 +5098,21 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>17:53:42</t>
+          <t>18:27:26</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>19:33</t>
+          <t>19:19</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>100</v>
+        <v>52</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,21 +5123,21 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>17:53:42</t>
+          <t>18:27:26</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5153,18 +5153,318 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
+          <t>19:22</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>89</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>18:27:26</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>56</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>18:27:26</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>19:26</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>59</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>17:53:42</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>19:33</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>100</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>18:27:26</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>73</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>18:27:26</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>19:41</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D198" t="n">
+        <v>74</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>18:27:26</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
           <t>19:43</t>
         </is>
       </c>
-      <c r="C193" t="inlineStr">
+      <c r="C199" t="inlineStr">
         <is>
           <t>81_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D193" t="n">
-        <v>110</v>
-      </c>
-      <c r="E193" t="inlineStr">
+      <c r="D199" t="n">
+        <v>76</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>18:27:26</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>19:54</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D200" t="n">
+        <v>87</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>18:27:26</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>20:01</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>94</v>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>18:27:26</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D202" t="n">
+        <v>95</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>18:27:26</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>20:03</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>96</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>18:27:26</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>20:23</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D204" t="n">
+        <v>116</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>18:27:26</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>20:25</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>118</v>
+      </c>
+      <c r="E205" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5181,7 +5481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5194,14 +5494,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:53:42</t>
+          <t>Última actualización: 18:27:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 31</t>
+          <t>Total filas: 34</t>
         </is>
       </c>
     </row>
@@ -5985,23 +6285,98 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>18:27:26</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>41</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>17:53:42</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>19:22</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D36" t="n">
+      <c r="D37" t="n">
         <v>89</v>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>18:27:26</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>56</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>18:27:26</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>20:03</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>96</v>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6018,7 +6393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6031,14 +6406,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:53:42</t>
+          <t>Última actualización: 18:27:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 27</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -6647,7 +7022,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>17:05:08</t>
+          <t>18:27:26</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -6661,7 +7036,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>85</v>
+        <v>3</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -6722,7 +7097,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>17:05:08</t>
+          <t>18:27:26</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -6736,11 +7111,36 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>117</v>
+        <v>35</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>18:27:26</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>95</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1919
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-24.xlsx
+++ b/data/horarios-141-2026-03-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E205"/>
+  <dimension ref="A1:E216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:27:26</t>
+          <t>Última actualización: 18:58:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 200</t>
+          <t>Total filas: 211</t>
         </is>
       </c>
     </row>
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>09:00:34</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>09:00:34</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>13:42:53</t>
+          <t>14:39:41</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>88</v>
+        <v>31</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>14:39:41</t>
+          <t>13:42:53</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>31</v>
+        <v>88</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -4398,7 +4398,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>17:05:08</t>
+          <t>16:36:44</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -4408,11 +4408,11 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>33</v>
+        <v>62</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,7 +4423,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>16:36:44</t>
+          <t>17:05:08</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -4433,11 +4433,11 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>62</v>
+        <v>33</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4948,12 +4948,12 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>18:27:26</t>
+          <t>18:58:51</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>19:04</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -4962,7 +4962,7 @@
         </is>
       </c>
       <c r="D185" t="n">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,21 +4973,21 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>17:53:42</t>
+          <t>18:27:26</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>19:07</t>
+          <t>19:05</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>74</v>
+        <v>38</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,12 +4998,12 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>18:27:26</t>
+          <t>18:58:51</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>19:07</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -5012,7 +5012,7 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>41</v>
+        <v>9</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,21 +5023,21 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>17:53:42</t>
+          <t>18:27:26</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>19:14</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>81</v>
+        <v>41</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,12 +5048,12 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>17:53:42</t>
+          <t>18:58:51</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:11</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -5062,7 +5062,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>84</v>
+        <v>13</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,12 +5073,12 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>18:27:26</t>
+          <t>17:53:42</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:14</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -5087,7 +5087,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>50</v>
+        <v>81</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,21 +5098,21 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>18:27:26</t>
+          <t>18:58:51</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>19:19</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5128,16 +5128,16 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5153,16 +5153,16 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>19:22</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5178,16 +5178,16 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:19</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5198,21 +5198,21 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>18:27:26</t>
+          <t>18:58:51</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>19:26</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>59</v>
+        <v>23</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,21 +5223,21 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>17:53:42</t>
+          <t>18:58:51</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>19:33</t>
+          <t>19:22</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>100</v>
+        <v>24</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5253,16 +5253,16 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>73</v>
+        <v>56</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,21 +5273,21 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>18:27:26</t>
+          <t>18:58:51</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>19:41</t>
+          <t>19:25</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>74</v>
+        <v>27</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5303,16 +5303,16 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>19:43</t>
+          <t>19:26</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>76</v>
+        <v>59</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,21 +5323,21 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>18:27:26</t>
+          <t>17:53:42</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>19:54</t>
+          <t>19:33</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,21 +5348,21 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>18:27:26</t>
+          <t>18:58:51</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>94</v>
+        <v>42</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,21 +5373,21 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>18:27:26</t>
+          <t>18:58:51</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>20:02</t>
+          <t>19:41</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>95</v>
+        <v>43</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5398,21 +5398,21 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>18:27:26</t>
+          <t>18:58:51</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>20:03</t>
+          <t>19:43</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>96</v>
+        <v>45</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5428,16 +5428,16 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>20:23</t>
+          <t>19:54</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>116</v>
+        <v>87</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5448,23 +5448,298 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
+          <t>18:58:51</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>19:55</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>57</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>18:58:51</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>20:01</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>63</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>18:58:51</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>64</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
           <t>18:27:26</t>
         </is>
       </c>
-      <c r="B205" t="inlineStr">
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>20:03</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>96</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>18:58:51</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>20:04</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>66</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>18:58:51</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>20:22</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>84</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>18:27:26</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>20:23</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D211" t="n">
+        <v>116</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>18:58:51</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>20:24</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>86</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>18:27:26</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
         <is>
           <t>20:25</t>
         </is>
       </c>
-      <c r="C205" t="inlineStr">
+      <c r="C213" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D205" t="n">
+      <c r="D213" t="n">
         <v>118</v>
       </c>
-      <c r="E205" t="inlineStr">
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>18:58:51</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D214" t="n">
+        <v>103</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>18:58:51</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>20:44</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D215" t="n">
+        <v>106</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>18:58:51</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D216" t="n">
+        <v>118</v>
+      </c>
+      <c r="E216" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5481,7 +5756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5494,14 +5769,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:27:26</t>
+          <t>Última actualización: 18:58:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 34</t>
+          <t>Total filas: 36</t>
         </is>
       </c>
     </row>
@@ -6260,7 +6535,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>17:53:42</t>
+          <t>18:58:51</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -6274,7 +6549,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>74</v>
+        <v>9</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -6310,7 +6585,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>17:53:42</t>
+          <t>18:58:51</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -6324,7 +6599,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>89</v>
+        <v>24</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -6377,6 +6652,56 @@
         <v>96</v>
       </c>
       <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>18:58:51</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>20:04</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>66</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>18:58:51</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>103</v>
+      </c>
+      <c r="E41" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6393,7 +6718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6406,14 +6731,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:27:26</t>
+          <t>Última actualización: 18:58:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 28</t>
+          <t>Total filas: 30</t>
         </is>
       </c>
     </row>
@@ -7072,7 +7397,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>17:53:42</t>
+          <t>18:58:51</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -7086,7 +7411,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>68</v>
+        <v>3</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -7122,23 +7447,73 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>18:58:51</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>20:01</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>63</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>18:27:26</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>20:02</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D33" t="n">
+      <c r="D34" t="n">
         <v>95</v>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>18:58:51</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>103</v>
+      </c>
+      <c r="E35" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1920
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-24.xlsx
+++ b/data/horarios-141-2026-03-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E216"/>
+  <dimension ref="A1:E227"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:58:51</t>
+          <t>Última actualización: 19:29:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 211</t>
+          <t>Total filas: 222</t>
         </is>
       </c>
     </row>
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>09:00:34</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>09:00:34</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>12:46:57</t>
+          <t>11:44:14</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>11</v>
+        <v>73</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>11:44:14</t>
+          <t>12:46:57</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2633,11 +2633,11 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>73</v>
+        <v>11</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>18:58:51</t>
+          <t>19:29:07</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5362,7 +5362,7 @@
         </is>
       </c>
       <c r="D201" t="n">
-        <v>42</v>
+        <v>11</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,7 +5373,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>18:58:51</t>
+          <t>19:29:07</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -5387,7 +5387,7 @@
         </is>
       </c>
       <c r="D202" t="n">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5398,7 +5398,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>18:58:51</t>
+          <t>19:29:07</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5412,7 +5412,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5448,7 +5448,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>18:58:51</t>
+          <t>19:29:07</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -5462,7 +5462,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,7 +5473,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>18:58:51</t>
+          <t>19:29:07</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -5487,7 +5487,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>63</v>
+        <v>32</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5548,21 +5548,21 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>18:58:51</t>
+          <t>19:29:07</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>20:04</t>
+          <t>20:03</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>66</v>
+        <v>34</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5578,16 +5578,16 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>20:22</t>
+          <t>20:04</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,21 +5598,21 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>18:27:26</t>
+          <t>19:29:07</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>20:23</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>116</v>
+        <v>36</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5628,16 +5628,16 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>20:24</t>
+          <t>20:22</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5653,16 +5653,16 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>20:25</t>
+          <t>20:23</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5678,16 +5678,16 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:24</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>103</v>
+        <v>86</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,21 +5698,21 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>18:58:51</t>
+          <t>19:29:07</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>20:44</t>
+          <t>20:25</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>106</v>
+        <v>56</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,23 +5723,298 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
+          <t>19:29:07</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>20:31</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D216" t="n">
+        <v>62</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
           <t>18:58:51</t>
         </is>
       </c>
-      <c r="B216" t="inlineStr">
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D217" t="n">
+        <v>103</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>19:29:07</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D218" t="n">
+        <v>73</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>18:58:51</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>20:44</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D219" t="n">
+        <v>106</v>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>19:29:07</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D220" t="n">
+        <v>76</v>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>19:29:07</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>20:50</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D221" t="n">
+        <v>81</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>19:29:07</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>20:51</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D222" t="n">
+        <v>82</v>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>19:29:07</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D223" t="n">
+        <v>86</v>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>18:58:51</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
         <is>
           <t>20:56</t>
         </is>
       </c>
-      <c r="C216" t="inlineStr">
+      <c r="C224" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D216" t="n">
+      <c r="D224" t="n">
         <v>118</v>
       </c>
-      <c r="E216" t="inlineStr">
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>19:29:07</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>21:03</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D225" t="n">
+        <v>94</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>19:29:07</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>21:10</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>101</v>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>19:29:07</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>21:26</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D227" t="n">
+        <v>117</v>
+      </c>
+      <c r="E227" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5756,7 +6031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5769,14 +6044,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:58:51</t>
+          <t>Última actualización: 19:29:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 36</t>
+          <t>Total filas: 38</t>
         </is>
       </c>
     </row>
@@ -6685,23 +6960,73 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>19:29:07</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>20:05</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>36</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>18:58:51</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>20:41</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D41" t="n">
+      <c r="D42" t="n">
         <v>103</v>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>19:29:07</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>73</v>
+      </c>
+      <c r="E43" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6718,7 +7043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6731,14 +7056,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:58:51</t>
+          <t>Última actualización: 19:29:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 30</t>
+          <t>Total filas: 31</t>
         </is>
       </c>
     </row>
@@ -7472,7 +7797,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>18:27:26</t>
+          <t>19:29:07</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -7486,7 +7811,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>95</v>
+        <v>33</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -7514,6 +7839,31 @@
         <v>103</v>
       </c>
       <c r="E35" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>19:29:07</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>73</v>
+      </c>
+      <c r="E36" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1921
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-24.xlsx
+++ b/data/horarios-141-2026-03-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E227"/>
+  <dimension ref="A1:E236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:29:07</t>
+          <t>Última actualización: 19:58:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 222</t>
+          <t>Total filas: 231</t>
         </is>
       </c>
     </row>
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>11:44:14</t>
+          <t>12:46:57</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>73</v>
+        <v>11</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>12:46:57</t>
+          <t>11:44:14</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2633,11 +2633,11 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>11</v>
+        <v>73</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>13:42:53</t>
+          <t>12:46:57</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>25</v>
+        <v>81</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>12:46:57</t>
+          <t>13:42:53</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>81</v>
+        <v>25</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -5523,21 +5523,21 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>18:27:26</t>
+          <t>19:58:04</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>20:03</t>
+          <t>20:02</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>96</v>
+        <v>4</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,7 +5548,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>19:29:07</t>
+          <t>18:27:26</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -5558,11 +5558,11 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>34</v>
+        <v>96</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5573,21 +5573,21 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>18:58:51</t>
+          <t>19:58:04</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>20:04</t>
+          <t>20:03</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>66</v>
+        <v>5</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,12 +5598,12 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>19:29:07</t>
+          <t>18:58:51</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>20:04</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -5612,7 +5612,7 @@
         </is>
       </c>
       <c r="D211" t="n">
-        <v>36</v>
+        <v>66</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,21 +5623,21 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>18:58:51</t>
+          <t>19:29:07</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>20:22</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>84</v>
+        <v>36</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,21 +5648,21 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>18:27:26</t>
+          <t>19:58:04</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>20:23</t>
+          <t>20:07</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>116</v>
+        <v>9</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5678,16 +5678,16 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>20:24</t>
+          <t>20:22</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,21 +5698,21 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>19:29:07</t>
+          <t>18:27:26</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>20:25</t>
+          <t>20:23</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>56</v>
+        <v>116</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,21 +5723,21 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>19:29:07</t>
+          <t>18:58:51</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>20:31</t>
+          <t>20:24</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>62</v>
+        <v>86</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,21 +5748,21 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>18:58:51</t>
+          <t>19:58:04</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:25</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>103</v>
+        <v>27</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5778,16 +5778,16 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>20:42</t>
+          <t>20:31</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,21 +5798,21 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>18:58:51</t>
+          <t>19:58:04</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>20:44</t>
+          <t>20:36</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>106</v>
+        <v>38</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,21 +5823,21 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>19:29:07</t>
+          <t>19:58:04</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>20:45</t>
+          <t>20:37</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>76</v>
+        <v>39</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5848,21 +5848,21 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>19:29:07</t>
+          <t>18:58:51</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>20:50</t>
+          <t>20:41</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>81</v>
+        <v>103</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5873,21 +5873,21 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>19:29:07</t>
+          <t>19:58:04</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>20:51</t>
+          <t>20:42</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>82</v>
+        <v>44</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,21 +5898,21 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>19:29:07</t>
+          <t>18:58:51</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>20:55</t>
+          <t>20:44</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>86</v>
+        <v>106</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,21 +5923,21 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>18:58:51</t>
+          <t>19:58:04</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>118</v>
+        <v>47</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5953,16 +5953,16 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>21:03</t>
+          <t>20:50</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>94</v>
+        <v>81</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5978,16 +5978,16 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>21:10</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>101</v>
+        <v>82</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,23 +5998,248 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
+          <t>19:58:04</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>20:52</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D227" t="n">
+        <v>54</v>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
           <t>19:29:07</t>
         </is>
       </c>
-      <c r="B227" t="inlineStr">
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
+        <v>86</v>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>18:58:51</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D229" t="n">
+        <v>118</v>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>19:58:04</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>20:57</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D230" t="n">
+        <v>59</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>19:58:04</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>21:03</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D231" t="n">
+        <v>65</v>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>19:58:04</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>21:10</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D232" t="n">
+        <v>72</v>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>19:58:04</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
         <is>
           <t>21:26</t>
         </is>
       </c>
-      <c r="C227" t="inlineStr">
+      <c r="C233" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D227" t="n">
-        <v>117</v>
-      </c>
-      <c r="E227" t="inlineStr">
+      <c r="D233" t="n">
+        <v>88</v>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>19:58:04</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D234" t="n">
+        <v>96</v>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>19:58:04</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D235" t="n">
+        <v>98</v>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>19:58:04</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>21:46</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D236" t="n">
+        <v>108</v>
+      </c>
+      <c r="E236" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6031,7 +6256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6044,14 +6269,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:29:07</t>
+          <t>Última actualización: 19:58:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 38</t>
+          <t>Total filas: 39</t>
         </is>
       </c>
     </row>
@@ -6985,21 +7210,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>18:58:51</t>
+          <t>19:58:04</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:07</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>103</v>
+        <v>9</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -7010,23 +7235,48 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>19:29:07</t>
+          <t>18:58:51</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>103</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>19:58:04</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
           <t>20:42</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D43" t="n">
-        <v>73</v>
-      </c>
-      <c r="E43" t="inlineStr">
+      <c r="D44" t="n">
+        <v>44</v>
+      </c>
+      <c r="E44" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7043,7 +7293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7056,14 +7306,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:29:07</t>
+          <t>Última actualización: 19:58:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 31</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -7772,12 +8022,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>18:58:51</t>
+          <t>19:58:04</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:59</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -7786,7 +8036,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>63</v>
+        <v>1</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -7797,12 +8047,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>19:29:07</t>
+          <t>18:58:51</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>20:02</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -7811,7 +8061,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>33</v>
+        <v>63</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -7822,12 +8072,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>18:58:51</t>
+          <t>19:29:07</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:02</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -7836,7 +8086,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>103</v>
+        <v>33</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -7847,23 +8097,48 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>19:29:07</t>
+          <t>18:58:51</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>103</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>19:58:04</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
           <t>20:42</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D36" t="n">
-        <v>73</v>
-      </c>
-      <c r="E36" t="inlineStr">
+      <c r="D37" t="n">
+        <v>44</v>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1922
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-24.xlsx
+++ b/data/horarios-141-2026-03-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E236"/>
+  <dimension ref="A1:E240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:58:04</t>
+          <t>Última actualización: 20:28:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 231</t>
+          <t>Total filas: 235</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>09:00:34</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>09:00:34</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -2008,7 +2008,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -2033,7 +2033,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>12:46:57</t>
+          <t>11:44:14</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>11</v>
+        <v>73</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>11:44:14</t>
+          <t>12:46:57</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2633,11 +2633,11 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>73</v>
+        <v>11</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>12:46:57</t>
+          <t>11:44:14</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>27</v>
+        <v>89</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>11:44:14</t>
+          <t>12:46:57</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>89</v>
+        <v>27</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -3783,7 +3783,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -5548,7 +5548,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>18:27:26</t>
+          <t>19:58:04</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -5558,11 +5558,11 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>96</v>
+        <v>5</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>19:58:04</t>
+          <t>18:27:26</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -5583,11 +5583,11 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>5</v>
+        <v>96</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5798,7 +5798,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>19:58:04</t>
+          <t>20:28:28</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -5812,7 +5812,7 @@
         </is>
       </c>
       <c r="D219" t="n">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,7 +5823,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>19:58:04</t>
+          <t>20:28:28</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -5837,7 +5837,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5848,7 +5848,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>18:58:51</t>
+          <t>20:28:28</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -5862,7 +5862,7 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>103</v>
+        <v>13</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5923,7 +5923,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>19:58:04</t>
+          <t>20:28:28</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -5937,7 +5937,7 @@
         </is>
       </c>
       <c r="D224" t="n">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5973,7 +5973,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>19:29:07</t>
+          <t>20:28:28</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -5987,7 +5987,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>82</v>
+        <v>23</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -6048,7 +6048,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>18:58:51</t>
+          <t>20:28:28</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -6062,7 +6062,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>118</v>
+        <v>28</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6098,12 +6098,12 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>19:58:04</t>
+          <t>20:28:28</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>21:03</t>
+          <t>21:02</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
@@ -6112,7 +6112,7 @@
         </is>
       </c>
       <c r="D231" t="n">
-        <v>65</v>
+        <v>34</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6128,16 +6128,16 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>21:10</t>
+          <t>21:03</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,21 +6148,21 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>19:58:04</t>
+          <t>20:28:28</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>21:26</t>
+          <t>21:10</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>88</v>
+        <v>42</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6173,21 +6173,21 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>19:58:04</t>
+          <t>20:28:28</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:26</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>96</v>
+        <v>58</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6198,21 +6198,21 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>19:58:04</t>
+          <t>20:28:28</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>21:36</t>
+          <t>21:34</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>98</v>
+        <v>66</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,23 +6223,123 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>19:58:04</t>
+          <t>20:28:28</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D236" t="n">
+        <v>68</v>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>20:28:28</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
           <t>21:46</t>
         </is>
       </c>
-      <c r="C236" t="inlineStr">
+      <c r="C237" t="inlineStr">
         <is>
           <t>14X44_ABASTO</t>
         </is>
       </c>
-      <c r="D236" t="n">
-        <v>108</v>
-      </c>
-      <c r="E236" t="inlineStr">
+      <c r="D237" t="n">
+        <v>78</v>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>20:28:28</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>21:51</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D238" t="n">
+        <v>83</v>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>20:28:28</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>22:04</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D239" t="n">
+        <v>96</v>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>20:28:28</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>22:13</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D240" t="n">
+        <v>105</v>
+      </c>
+      <c r="E240" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6269,7 +6369,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:58:04</t>
+          <t>Última actualización: 20:28:28</t>
         </is>
       </c>
     </row>
@@ -7235,7 +7335,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>18:58:51</t>
+          <t>20:28:28</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -7249,7 +7349,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>103</v>
+        <v>13</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -7293,7 +7393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7306,14 +7406,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:58:04</t>
+          <t>Última actualización: 20:28:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 32</t>
+          <t>Total filas: 35</t>
         </is>
       </c>
     </row>
@@ -8141,6 +8241,81 @@
       <c r="E37" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>20:28:28</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>20:44</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>16</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>20:28:28</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>21:26</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>58</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>20:28:28</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>22:16</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>108</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1923
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-24.xlsx
+++ b/data/horarios-141-2026-03-24.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E240"/>
+  <dimension ref="A1:E246"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:28:28</t>
+          <t>Última actualización: 20:54:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 235</t>
+          <t>Total filas: 241</t>
         </is>
       </c>
     </row>
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08:24:08</t>
+          <t>09:00:34</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1333,11 +1333,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>09:00:34</t>
+          <t>08:24:08</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1358,11 +1358,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -2008,7 +2008,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -2033,7 +2033,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>12:46:57</t>
+          <t>13:42:53</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>81</v>
+        <v>25</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>13:42:53</t>
+          <t>12:46:57</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>25</v>
+        <v>81</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3783,7 +3783,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -4058,7 +4058,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -4083,7 +4083,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -4398,7 +4398,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>16:36:44</t>
+          <t>17:05:08</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -4408,11 +4408,11 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>62</v>
+        <v>33</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,7 +4423,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>17:05:08</t>
+          <t>16:36:44</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -4433,11 +4433,11 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>33</v>
+        <v>62</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -5548,7 +5548,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>19:58:04</t>
+          <t>18:27:26</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -5558,11 +5558,11 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>5</v>
+        <v>96</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>18:27:26</t>
+          <t>19:58:04</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -5583,11 +5583,11 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>96</v>
+        <v>5</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -6048,7 +6048,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>20:28:28</t>
+          <t>20:54:26</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -6062,7 +6062,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>19:58:04</t>
+          <t>20:54:26</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6137,7 +6137,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>65</v>
+        <v>9</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,7 +6148,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>20:28:28</t>
+          <t>20:54:26</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -6162,7 +6162,7 @@
         </is>
       </c>
       <c r="D233" t="n">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6173,7 +6173,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>20:28:28</t>
+          <t>20:54:26</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -6187,7 +6187,7 @@
         </is>
       </c>
       <c r="D234" t="n">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6198,7 +6198,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>20:28:28</t>
+          <t>20:54:26</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -6212,7 +6212,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>66</v>
+        <v>40</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,7 +6223,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>20:28:28</t>
+          <t>20:54:26</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -6237,7 +6237,7 @@
         </is>
       </c>
       <c r="D236" t="n">
-        <v>68</v>
+        <v>42</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6248,21 +6248,21 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>20:28:28</t>
+          <t>20:54:26</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>21:46</t>
+          <t>21:40</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D237" t="n">
-        <v>78</v>
+        <v>46</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -6273,21 +6273,21 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>20:28:28</t>
+          <t>20:54:26</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>21:51</t>
+          <t>21:46</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>83</v>
+        <v>52</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -6303,16 +6303,16 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>22:04</t>
+          <t>21:51</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6323,23 +6323,173 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
+          <t>20:54:26</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>22:04</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D240" t="n">
+        <v>70</v>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>20:54:26</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>22:11</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D241" t="n">
+        <v>77</v>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
           <t>20:28:28</t>
         </is>
       </c>
-      <c r="B240" t="inlineStr">
+      <c r="B242" t="inlineStr">
         <is>
           <t>22:13</t>
         </is>
       </c>
-      <c r="C240" t="inlineStr">
+      <c r="C242" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D240" t="n">
+      <c r="D242" t="n">
         <v>105</v>
       </c>
-      <c r="E240" t="inlineStr">
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>20:54:26</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D243" t="n">
+        <v>96</v>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>20:54:26</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>22:33</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D244" t="n">
+        <v>99</v>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>20:54:26</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>22:36</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D245" t="n">
+        <v>102</v>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>20:54:26</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>22:43</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D246" t="n">
+        <v>109</v>
+      </c>
+      <c r="E246" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6356,7 +6506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6369,14 +6519,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:28:28</t>
+          <t>Última actualización: 20:54:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 39</t>
+          <t>Total filas: 40</t>
         </is>
       </c>
     </row>
@@ -7377,6 +7527,31 @@
         <v>44</v>
       </c>
       <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>20:54:26</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>22:33</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>99</v>
+      </c>
+      <c r="E45" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7406,7 +7581,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:28:28</t>
+          <t>Última actualización: 20:54:26</t>
         </is>
       </c>
     </row>
@@ -8272,7 +8447,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>20:28:28</t>
+          <t>20:54:26</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -8286,7 +8461,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -8297,7 +8472,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>20:28:28</t>
+          <t>20:54:26</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -8311,7 +8486,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>108</v>
+        <v>82</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>

</xml_diff>